<commit_message>
all modules, test script ready
</commit_message>
<xml_diff>
--- a/src/test/resources/ninzaHRM.xlsx
+++ b/src/test/resources/ninzaHRM.xlsx
@@ -3,22 +3,23 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\shashank\Capgemini_Training\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\shashank\Capgemini_Training\ninza-sprint\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F39B0E81-7942-4D92-ABCF-D2E795733245}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59C64E8E-A137-4868-B49F-D3785B96F241}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{62126B80-DC88-4390-B360-29F3B85AC0F5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{62126B80-DC88-4390-B360-29F3B85AC0F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
   <si>
     <t>username</t>
   </si>
@@ -41,12 +42,73 @@
   </si>
   <si>
     <t xml:space="preserve">sha </t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">email </t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>designation</t>
+  </si>
+  <si>
+    <t>experience</t>
+  </si>
+  <si>
+    <t>shank</t>
+  </si>
+  <si>
+    <t>shank@gmail.com</t>
+  </si>
+  <si>
+    <t>shank@1234</t>
+  </si>
+  <si>
+    <t>CEO</t>
+  </si>
+  <si>
+    <t>project</t>
+  </si>
+  <si>
+    <t>TP</t>
+  </si>
+  <si>
+    <t>shank@1234-14201161</t>
+  </si>
+  <si>
+    <t>shank@1234-14201161347818543</t>
+  </si>
+  <si>
+    <t>shank@1234-14201161347818543877752222</t>
+  </si>
+  <si>
+    <t>shank@1234-14201161347818543877752222514190763</t>
+  </si>
+  <si>
+    <t>shank@1234-142011613478185438777522225141907631245586902</t>
+  </si>
+  <si>
+    <t>shank@1234-142011613478185438777522225141907631245586902994490572</t>
+  </si>
+  <si>
+    <t>shank@1234-142011613478185438777522225141907631245586902994490572-921774580</t>
+  </si>
+  <si>
+    <t>shank@1234-142011613478185438777522225141907631245586902994490572-921774580400318700</t>
+  </si>
+  <si>
+    <t>shank@1234-142011613478185438777522225141907631245586902994490572-921774580400318700-752918855</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -406,20 +468,20 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.109375" customWidth="1"/>
-    <col min="2" max="2" width="19.33203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="15.109375"/>
+    <col min="2" max="2" customWidth="true" width="19.33203125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -439,20 +501,20 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.109375" customWidth="1"/>
-    <col min="2" max="2" width="17.44140625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="17.109375"/>
+    <col min="2" max="2" customWidth="true" width="17.44140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -460,20 +522,20 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" t="s" s="0">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" t="s" s="0">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B6" t="s">
+      <c r="B6" t="s" s="0">
         <v>3</v>
       </c>
     </row>
@@ -483,4 +545,72 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5E10EE1-9790-4EC9-A8E2-E040B7E41456}">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" customWidth="true" width="13.88671875"/>
+    <col min="2" max="2" customWidth="true" width="16.0"/>
+    <col min="3" max="3" customWidth="true" width="19.77734375"/>
+    <col min="4" max="4" customWidth="true" width="17.44140625"/>
+    <col min="5" max="5" customWidth="true" width="17.5546875"/>
+    <col min="6" max="6" customWidth="true" width="14.33203125"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="0">
+        <v>1234567890</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F2" s="0">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{7CF794C8-FB7F-409C-8393-4CA6320C95BC}"/>
+    <hyperlink ref="D2" r:id="rId2" xr:uid="{5AEDF1C6-9180-447C-8FC2-6AFA8F074FB1}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>